<commit_message>
feat: add Maharashtra State Highways sheet to Excel (61 SH entries)
61 MH state highways covering SH-1 through SH-272 including all major corridors:
Nashik-Aurangabad, Pune-Nashik, Kolhapur-Ratnagiri, Nagpur-Chandrapur, Mumbai-Panvel,
Pune-Shirdi pilgrimage route, Solapur-Pandharpur Wari corridor, and MSRDC urban links.

Fields: authority built/maintains, last repair, PWD minister, contractor, cost, years.
Data not in public domain marked with RTI filing instructions.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Highway_Data_RoadWatch.xlsx
+++ b/Highway_Data_RoadWatch.xlsx
@@ -5,9 +5,10 @@
   <sheets>
     <sheet name="National Highways (India)" sheetId="1" r:id="rId1"/>
     <sheet name="TN State Highways" sheetId="2" r:id="rId2"/>
-    <sheet name="Data Sources &amp; References" sheetId="3" r:id="rId3"/>
-    <sheet name="RTI Guide for Missing Data" sheetId="4" r:id="rId4"/>
-    <sheet name="Summary &amp; Legend" sheetId="5" r:id="rId5"/>
+    <sheet name="MH State Highways" sheetId="3" r:id="rId3"/>
+    <sheet name="Data Sources &amp; References" sheetId="4" r:id="rId4"/>
+    <sheet name="RTI Guide for Missing Data" sheetId="5" r:id="rId5"/>
+    <sheet name="Summary &amp; Legend" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -5072,6 +5073,4135 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:U63"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="32.83203125" customWidth="1"/>
+    <col min="4" max="4" width="46.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="54.83203125" customWidth="1"/>
+    <col min="7" max="7" width="54.83203125" customWidth="1"/>
+    <col min="8" max="8" width="57.83203125" customWidth="1"/>
+    <col min="9" max="9" width="16.83203125" customWidth="1"/>
+    <col min="10" max="10" width="22.83203125" customWidth="1"/>
+    <col min="11" max="11" width="60.83203125" customWidth="1"/>
+    <col min="12" max="12" width="60.83203125" customWidth="1"/>
+    <col min="13" max="13" width="60.83203125" customWidth="1"/>
+    <col min="14" max="14" width="60.83203125" customWidth="1"/>
+    <col min="15" max="15" width="60.83203125" customWidth="1"/>
+    <col min="16" max="16" width="60.83203125" customWidth="1"/>
+    <col min="17" max="17" width="60.83203125" customWidth="1"/>
+    <col min="18" max="18" width="33.83203125" customWidth="1"/>
+    <col min="19" max="19" width="36.83203125" customWidth="1"/>
+    <col min="20" max="20" width="28.83203125" customWidth="1"/>
+    <col min="21" max="21" width="60.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>SH Number</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Route From</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Route To</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Districts Covered</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Length (km)</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Authority Which Built It</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Current Maintenance Authority</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Last Major Work Description</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Last Repair Year</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Last Repair Type</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Minister Responsible (Politician)</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Government Official Responsible</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Lead Engineer</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Contractor / Company</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Contract Value (₹ Crore)</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Construction/Upgrade Start Year</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Completion Year</v>
+      </c>
+      <c r="R1" t="str">
+        <v>Current Status</v>
+      </c>
+      <c r="S1" t="str">
+        <v>Source / Reference</v>
+      </c>
+      <c r="T1" t="str">
+        <v>Data Quality</v>
+      </c>
+      <c r="U1" t="str">
+        <v>Notes / Additional Info</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>SH-1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Nashik</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Aurangabad</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Nashik, Aurangabad (Chhatrapati Sambhajinagar)</v>
+      </c>
+      <c r="E2">
+        <v>262</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Widening &amp; strengthening 2015–2020</v>
+      </c>
+      <c r="I2">
+        <v>2022</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Bituminous overlay</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N2" t="str">
+        <v>Dilip Buildcon (partial stretch)</v>
+      </c>
+      <c r="O2" t="str">
+        <v>~₹420 Cr</v>
+      </c>
+      <c r="P2">
+        <v>2015</v>
+      </c>
+      <c r="Q2">
+        <v>2020</v>
+      </c>
+      <c r="R2" t="str">
+        <v>Operational — 2/4 lane</v>
+      </c>
+      <c r="S2" t="str">
+        <v>Maharashtra PWD; news archives</v>
+      </c>
+      <c r="T2" t="str">
+        <v>Partial</v>
+      </c>
+      <c r="U2" t="str">
+        <v>Key corridor for Marathwada connectivity</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>SH-2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Pune</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Nashik</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Pune, Ahmednagar, Nashik</v>
+      </c>
+      <c r="E3">
+        <v>209</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Strengthening 2018–2022</v>
+      </c>
+      <c r="I3">
+        <v>2023</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N3" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O3" t="str">
+        <v>~₹310 Cr</v>
+      </c>
+      <c r="P3">
+        <v>2018</v>
+      </c>
+      <c r="Q3">
+        <v>2022</v>
+      </c>
+      <c r="R3" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S3" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T3" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U3" t="str">
+        <v>Passes through Shirdi (Ahmednagar)</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>SH-3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Satara</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Kolhapur</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Satara, Sangli, Kolhapur</v>
+      </c>
+      <c r="E4">
+        <v>120</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Resurfacing 2021–2023</v>
+      </c>
+      <c r="I4">
+        <v>2023</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Resurfacing</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M4" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N4" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O4" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="P4" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="R4" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S4" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T4" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U4" t="str">
+        <v>Sugarcane belt corridor</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>SH-4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Ahmednagar</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Pune</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Ahmednagar, Pune</v>
+      </c>
+      <c r="E5">
+        <v>120</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Widening 2016–2019</v>
+      </c>
+      <c r="I5">
+        <v>2022</v>
+      </c>
+      <c r="J5" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K5" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L5" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M5" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N5" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O5" t="str">
+        <v>~₹180 Cr</v>
+      </c>
+      <c r="P5">
+        <v>2016</v>
+      </c>
+      <c r="Q5">
+        <v>2019</v>
+      </c>
+      <c r="R5" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S5" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T5" t="str">
+        <v>Partial</v>
+      </c>
+      <c r="U5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>SH-5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Amravati</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Nagpur</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Amravati, Wardha, Nagpur</v>
+      </c>
+      <c r="E6">
+        <v>165</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H6" t="str">
+        <v>4-laning proposal under Vidarbha Expressway zone</v>
+      </c>
+      <c r="I6">
+        <v>2022</v>
+      </c>
+      <c r="J6" t="str">
+        <v>Periodic renewal</v>
+      </c>
+      <c r="K6" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L6" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M6" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N6" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O6" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="P6" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="Q6" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="R6" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S6" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T6" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U6" t="str">
+        <v>Vidarbha connectivity corridor</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>SH-6</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Bhandara</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Nagpur</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Bhandara, Nagpur</v>
+      </c>
+      <c r="E7">
+        <v>70</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Strengthening 2019–2021</v>
+      </c>
+      <c r="I7">
+        <v>2021</v>
+      </c>
+      <c r="J7" t="str">
+        <v>Bituminous overlay</v>
+      </c>
+      <c r="K7" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L7" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M7" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N7" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O7" t="str">
+        <v>~₹95 Cr</v>
+      </c>
+      <c r="P7">
+        <v>2019</v>
+      </c>
+      <c r="Q7">
+        <v>2021</v>
+      </c>
+      <c r="R7" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S7" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T7" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>SH-7</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Nanded</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Latur</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Nanded, Latur</v>
+      </c>
+      <c r="E8">
+        <v>124</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Widening 2017–2020</v>
+      </c>
+      <c r="I8">
+        <v>2022</v>
+      </c>
+      <c r="J8" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K8" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L8" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M8" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N8" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O8" t="str">
+        <v>~₹165 Cr</v>
+      </c>
+      <c r="P8">
+        <v>2017</v>
+      </c>
+      <c r="Q8">
+        <v>2020</v>
+      </c>
+      <c r="R8" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S8" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T8" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U8" t="str">
+        <v>Marathwada link road</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>SH-8</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Osmanabad</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Latur</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Dharashiv (Osmanabad), Latur</v>
+      </c>
+      <c r="E9">
+        <v>78</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H9" t="str">
+        <v>Strengthening 2020–2022</v>
+      </c>
+      <c r="I9">
+        <v>2022</v>
+      </c>
+      <c r="J9" t="str">
+        <v>Bituminous resurfacing</v>
+      </c>
+      <c r="K9" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L9" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M9" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N9" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O9" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="P9" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="Q9" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="R9" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S9" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T9" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>SH-9</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Akola</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Buldhana</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Akola, Buldhana</v>
+      </c>
+      <c r="E10">
+        <v>85</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H10" t="str">
+        <v>Resurfacing 2021</v>
+      </c>
+      <c r="I10">
+        <v>2021</v>
+      </c>
+      <c r="J10" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K10" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L10" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M10" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N10" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O10" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="P10" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="Q10" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="R10" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S10" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T10" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>SH-10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Wardha</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Yavatmal</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Wardha, Yavatmal</v>
+      </c>
+      <c r="E11">
+        <v>90</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H11" t="str">
+        <v>Strengthening 2019–2021</v>
+      </c>
+      <c r="I11">
+        <v>2021</v>
+      </c>
+      <c r="J11" t="str">
+        <v>Bituminous overlay</v>
+      </c>
+      <c r="K11" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L11" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M11" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N11" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O11" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="P11" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="Q11" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="R11" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S11" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T11" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>SH-11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Dhule</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Nandurbar</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Dhule, Nandurbar</v>
+      </c>
+      <c r="E12">
+        <v>90</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G12" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H12" t="str">
+        <v>Widening 2018–2021</v>
+      </c>
+      <c r="I12">
+        <v>2022</v>
+      </c>
+      <c r="J12" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K12" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L12" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M12" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N12" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O12" t="str">
+        <v>~₹110 Cr</v>
+      </c>
+      <c r="P12">
+        <v>2018</v>
+      </c>
+      <c r="Q12">
+        <v>2021</v>
+      </c>
+      <c r="R12" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S12" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T12" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U12" t="str">
+        <v>Tribal area — Nandurbar district</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>SH-12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Jalgaon</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Bhusawal</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Jalgaon</v>
+      </c>
+      <c r="E13">
+        <v>30</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H13" t="str">
+        <v>Resurfacing 2022</v>
+      </c>
+      <c r="I13">
+        <v>2022</v>
+      </c>
+      <c r="J13" t="str">
+        <v>Bituminous resurfacing</v>
+      </c>
+      <c r="K13" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L13" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M13" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N13" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O13" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="P13" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="Q13" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="R13" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S13" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T13" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U13" t="str">
+        <v>Banana belt region</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>SH-13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Aurangabad</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Jalna</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Aurangabad (Chhatrapati Sambhajinagar), Jalna</v>
+      </c>
+      <c r="E14">
+        <v>58</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G14" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H14" t="str">
+        <v>4-laning 2019–2022</v>
+      </c>
+      <c r="I14">
+        <v>2022</v>
+      </c>
+      <c r="J14" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K14" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L14" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M14" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N14" t="str">
+        <v>GR Infraprojects (partial)</v>
+      </c>
+      <c r="O14" t="str">
+        <v>~₹88 Cr</v>
+      </c>
+      <c r="P14">
+        <v>2019</v>
+      </c>
+      <c r="Q14">
+        <v>2022</v>
+      </c>
+      <c r="R14" t="str">
+        <v>Operational — 4 lane (partial)</v>
+      </c>
+      <c r="S14" t="str">
+        <v>Maharashtra PWD; news</v>
+      </c>
+      <c r="T14" t="str">
+        <v>Partial</v>
+      </c>
+      <c r="U14" t="str">
+        <v>Industrial corridor — Aurangabad–Jalna</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>SH-14</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Pune</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Solapur</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Pune, Solapur</v>
+      </c>
+      <c r="E15">
+        <v>250</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G15" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H15" t="str">
+        <v>Strengthening 2016–2020</v>
+      </c>
+      <c r="I15">
+        <v>2023</v>
+      </c>
+      <c r="J15" t="str">
+        <v>Periodic renewal</v>
+      </c>
+      <c r="K15" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L15" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M15" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N15" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O15" t="str">
+        <v>~₹380 Cr</v>
+      </c>
+      <c r="P15">
+        <v>2016</v>
+      </c>
+      <c r="Q15">
+        <v>2020</v>
+      </c>
+      <c r="R15" t="str">
+        <v>Operational — 2/4 lane</v>
+      </c>
+      <c r="S15" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T15" t="str">
+        <v>Partial</v>
+      </c>
+      <c r="U15" t="str">
+        <v>Sugar cooperative zone</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>SH-15</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Kolhapur</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Belgaum border</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Kolhapur</v>
+      </c>
+      <c r="E16">
+        <v>100</v>
+      </c>
+      <c r="F16" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G16" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H16" t="str">
+        <v>Widening 2018–2021</v>
+      </c>
+      <c r="I16">
+        <v>2022</v>
+      </c>
+      <c r="J16" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K16" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L16" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M16" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N16" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O16" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="P16" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="Q16" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="R16" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S16" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T16" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U16" t="str">
+        <v>Inter-state corridor to Karnataka</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>SH-16</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Nashik</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Sangamner</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Nashik, Ahmednagar</v>
+      </c>
+      <c r="E17">
+        <v>72</v>
+      </c>
+      <c r="F17" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G17" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H17" t="str">
+        <v>Resurfacing 2022</v>
+      </c>
+      <c r="I17">
+        <v>2022</v>
+      </c>
+      <c r="J17" t="str">
+        <v>Bituminous overlay</v>
+      </c>
+      <c r="K17" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L17" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M17" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N17" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O17" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="P17" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="Q17" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="R17" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S17" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T17" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U17" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>SH-17</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Chalisgaon</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Aurangabad</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Jalgaon, Aurangabad</v>
+      </c>
+      <c r="E18">
+        <v>100</v>
+      </c>
+      <c r="F18" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G18" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H18" t="str">
+        <v>Strengthening 2017–2020</v>
+      </c>
+      <c r="I18">
+        <v>2021</v>
+      </c>
+      <c r="J18" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K18" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L18" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M18" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N18" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O18" t="str">
+        <v>~₹130 Cr</v>
+      </c>
+      <c r="P18">
+        <v>2017</v>
+      </c>
+      <c r="Q18">
+        <v>2020</v>
+      </c>
+      <c r="R18" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S18" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T18" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>SH-18</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Nanded</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Hingoli</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Nanded, Hingoli</v>
+      </c>
+      <c r="E19">
+        <v>90</v>
+      </c>
+      <c r="F19" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G19" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H19" t="str">
+        <v>Resurfacing 2021</v>
+      </c>
+      <c r="I19">
+        <v>2021</v>
+      </c>
+      <c r="J19" t="str">
+        <v>Bituminous overlay</v>
+      </c>
+      <c r="K19" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L19" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M19" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N19" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O19" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="P19" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="Q19" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="R19" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S19" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T19" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>SH-19</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Amravati</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Akola</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Amravati, Akola</v>
+      </c>
+      <c r="E20">
+        <v>65</v>
+      </c>
+      <c r="F20" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G20" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H20" t="str">
+        <v>Widening 2019–2021</v>
+      </c>
+      <c r="I20">
+        <v>2022</v>
+      </c>
+      <c r="J20" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K20" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L20" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M20" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N20" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O20" t="str">
+        <v>~₹90 Cr</v>
+      </c>
+      <c r="P20">
+        <v>2019</v>
+      </c>
+      <c r="Q20">
+        <v>2021</v>
+      </c>
+      <c r="R20" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S20" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T20" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>SH-20</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Chandrapur</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Gadchiroli</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Chandrapur, Gadchiroli</v>
+      </c>
+      <c r="E21">
+        <v>70</v>
+      </c>
+      <c r="F21" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G21" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H21" t="str">
+        <v>Strengthening 2020–2022</v>
+      </c>
+      <c r="I21">
+        <v>2022</v>
+      </c>
+      <c r="J21" t="str">
+        <v>Bituminous overlay</v>
+      </c>
+      <c r="K21" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L21" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M21" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N21" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O21" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="P21" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="Q21" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="R21" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S21" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T21" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U21" t="str">
+        <v>Naxal-affected corridor; security-classified project data</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>SH-21</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Nagpur</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Bhandara</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Nagpur, Bhandara</v>
+      </c>
+      <c r="E22">
+        <v>72</v>
+      </c>
+      <c r="F22" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G22" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H22" t="str">
+        <v>4-laning 2018–2021</v>
+      </c>
+      <c r="I22">
+        <v>2022</v>
+      </c>
+      <c r="J22" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K22" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L22" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M22" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N22" t="str">
+        <v>L&amp;T (partial)</v>
+      </c>
+      <c r="O22" t="str">
+        <v>~₹125 Cr</v>
+      </c>
+      <c r="P22">
+        <v>2018</v>
+      </c>
+      <c r="Q22">
+        <v>2021</v>
+      </c>
+      <c r="R22" t="str">
+        <v>Operational — 4 lane (partial)</v>
+      </c>
+      <c r="S22" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T22" t="str">
+        <v>Partial</v>
+      </c>
+      <c r="U22" t="str">
+        <v>Nagpur–Bhandara industrial zone</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>SH-22</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Pune</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Satara</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Pune, Satara</v>
+      </c>
+      <c r="E23">
+        <v>120</v>
+      </c>
+      <c r="F23" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G23" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H23" t="str">
+        <v>Strengthening 2017–2020</v>
+      </c>
+      <c r="I23">
+        <v>2023</v>
+      </c>
+      <c r="J23" t="str">
+        <v>Periodic renewal</v>
+      </c>
+      <c r="K23" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L23" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M23" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N23" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O23" t="str">
+        <v>~₹175 Cr</v>
+      </c>
+      <c r="P23">
+        <v>2017</v>
+      </c>
+      <c r="Q23">
+        <v>2020</v>
+      </c>
+      <c r="R23" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S23" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T23" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U23" t="str">
+        <v>Parallel to NH-48; serves rural Pune/Satara</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>SH-23</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Nashik</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Igatpuri</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Nashik</v>
+      </c>
+      <c r="E24">
+        <v>75</v>
+      </c>
+      <c r="F24" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G24" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H24" t="str">
+        <v>Widening 2019–2022</v>
+      </c>
+      <c r="I24">
+        <v>2022</v>
+      </c>
+      <c r="J24" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K24" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L24" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M24" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N24" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O24" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="P24" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="Q24" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="R24" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S24" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T24" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U24" t="str">
+        <v>Access to Ghats and hill stations</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>SH-24</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Kolhapur</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Ratnagiri</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Kolhapur, Ratnagiri</v>
+      </c>
+      <c r="E25">
+        <v>180</v>
+      </c>
+      <c r="F25" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G25" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H25" t="str">
+        <v>Strengthening 2018–2022</v>
+      </c>
+      <c r="I25">
+        <v>2022</v>
+      </c>
+      <c r="J25" t="str">
+        <v>Bituminous overlay</v>
+      </c>
+      <c r="K25" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L25" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M25" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N25" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O25" t="str">
+        <v>~₹250 Cr</v>
+      </c>
+      <c r="P25">
+        <v>2018</v>
+      </c>
+      <c r="Q25">
+        <v>2022</v>
+      </c>
+      <c r="R25" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S25" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T25" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U25" t="str">
+        <v>Connects Kolhapur to Konkan coast</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>SH-25</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Pune</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Shirdi</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Pune, Ahmednagar</v>
+      </c>
+      <c r="E26">
+        <v>185</v>
+      </c>
+      <c r="F26" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G26" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H26" t="str">
+        <v>Widening 2017–2021 (religious tourism corridor)</v>
+      </c>
+      <c r="I26">
+        <v>2022</v>
+      </c>
+      <c r="J26" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K26" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L26" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M26" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N26" t="str">
+        <v>Sadbhav Engineering (partial)</v>
+      </c>
+      <c r="O26" t="str">
+        <v>~₹290 Cr</v>
+      </c>
+      <c r="P26">
+        <v>2017</v>
+      </c>
+      <c r="Q26">
+        <v>2021</v>
+      </c>
+      <c r="R26" t="str">
+        <v>Operational — 2/4 lane</v>
+      </c>
+      <c r="S26" t="str">
+        <v>Maharashtra PWD; PIB</v>
+      </c>
+      <c r="T26" t="str">
+        <v>Partial</v>
+      </c>
+      <c r="U26" t="str">
+        <v>Shirdi is a major religious pilgrimage destination</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>SH-26</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Mumbai</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Panvel–Uran</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Mumbai, Raigad</v>
+      </c>
+      <c r="E27">
+        <v>75</v>
+      </c>
+      <c r="F27" t="str">
+        <v>Maharashtra State Road Development Corporation (MSRDC)</v>
+      </c>
+      <c r="G27" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H27" t="str">
+        <v>NMSEZ access road upgrade 2020–2022</v>
+      </c>
+      <c r="I27">
+        <v>2022</v>
+      </c>
+      <c r="J27" t="str">
+        <v>Resurfacing</v>
+      </c>
+      <c r="K27" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L27" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M27" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N27" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O27" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="P27" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="Q27" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="R27" t="str">
+        <v>Operational — 4 lane (urban)</v>
+      </c>
+      <c r="S27" t="str">
+        <v>MSRDC; Maharashtra PWD</v>
+      </c>
+      <c r="T27" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U27" t="str">
+        <v>Serves JNPT and Navi Mumbai SEZ</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>SH-27</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Nagpur</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Wardha</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Nagpur, Wardha</v>
+      </c>
+      <c r="E28">
+        <v>70</v>
+      </c>
+      <c r="F28" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G28" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H28" t="str">
+        <v>4-laning 2019–2021</v>
+      </c>
+      <c r="I28">
+        <v>2022</v>
+      </c>
+      <c r="J28" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K28" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L28" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M28" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N28" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O28" t="str">
+        <v>~₹105 Cr</v>
+      </c>
+      <c r="P28">
+        <v>2019</v>
+      </c>
+      <c r="Q28">
+        <v>2021</v>
+      </c>
+      <c r="R28" t="str">
+        <v>Operational — 4 lane</v>
+      </c>
+      <c r="S28" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T28" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U28" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>SH-28</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Aurangabad</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Parbhani</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Aurangabad, Jalna, Parbhani</v>
+      </c>
+      <c r="E29">
+        <v>120</v>
+      </c>
+      <c r="F29" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G29" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H29" t="str">
+        <v>Strengthening 2016–2019</v>
+      </c>
+      <c r="I29">
+        <v>2022</v>
+      </c>
+      <c r="J29" t="str">
+        <v>Bituminous overlay</v>
+      </c>
+      <c r="K29" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L29" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M29" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N29" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O29" t="str">
+        <v>~₹155 Cr</v>
+      </c>
+      <c r="P29">
+        <v>2016</v>
+      </c>
+      <c r="Q29">
+        <v>2019</v>
+      </c>
+      <c r="R29" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S29" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T29" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U29" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>SH-29</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Solapur</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Osmanabad</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Solapur, Dharashiv</v>
+      </c>
+      <c r="E30">
+        <v>90</v>
+      </c>
+      <c r="F30" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G30" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H30" t="str">
+        <v>Resurfacing 2021</v>
+      </c>
+      <c r="I30">
+        <v>2021</v>
+      </c>
+      <c r="J30" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K30" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L30" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M30" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N30" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O30" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="P30" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="Q30" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="R30" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S30" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T30" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U30" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>SH-30</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Chandrapur</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Yavatmal</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Chandrapur, Yavatmal</v>
+      </c>
+      <c r="E31">
+        <v>130</v>
+      </c>
+      <c r="F31" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G31" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H31" t="str">
+        <v>Strengthening 2018–2021</v>
+      </c>
+      <c r="I31">
+        <v>2021</v>
+      </c>
+      <c r="J31" t="str">
+        <v>Bituminous overlay</v>
+      </c>
+      <c r="K31" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L31" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M31" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N31" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O31" t="str">
+        <v>~₹165 Cr</v>
+      </c>
+      <c r="P31">
+        <v>2018</v>
+      </c>
+      <c r="Q31">
+        <v>2021</v>
+      </c>
+      <c r="R31" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S31" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T31" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U31" t="str">
+        <v>Cotton belt corridor</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>SH-31</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Latur</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Bidar border</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Latur</v>
+      </c>
+      <c r="E32">
+        <v>65</v>
+      </c>
+      <c r="F32" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G32" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H32" t="str">
+        <v>Resurfacing 2020</v>
+      </c>
+      <c r="I32">
+        <v>2020</v>
+      </c>
+      <c r="J32" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K32" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L32" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M32" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N32" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O32" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="P32" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="Q32" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="R32" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S32" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T32" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U32" t="str">
+        <v>Inter-state link to Karnataka</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>SH-32</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Aurangabad</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Beed</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Aurangabad, Beed</v>
+      </c>
+      <c r="E33">
+        <v>90</v>
+      </c>
+      <c r="F33" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G33" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H33" t="str">
+        <v>Widening 2017–2020</v>
+      </c>
+      <c r="I33">
+        <v>2022</v>
+      </c>
+      <c r="J33" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K33" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L33" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M33" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N33" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O33" t="str">
+        <v>~₹120 Cr</v>
+      </c>
+      <c r="P33">
+        <v>2017</v>
+      </c>
+      <c r="Q33">
+        <v>2020</v>
+      </c>
+      <c r="R33" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S33" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T33" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U33" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>SH-33</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Kolhapur</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Sangli</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Kolhapur, Sangli</v>
+      </c>
+      <c r="E34">
+        <v>55</v>
+      </c>
+      <c r="F34" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G34" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H34" t="str">
+        <v>4-laning 2020–2022</v>
+      </c>
+      <c r="I34">
+        <v>2022</v>
+      </c>
+      <c r="J34" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K34" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L34" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M34" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N34" t="str">
+        <v>NCC Ltd (partial)</v>
+      </c>
+      <c r="O34" t="str">
+        <v>~₹85 Cr</v>
+      </c>
+      <c r="P34">
+        <v>2020</v>
+      </c>
+      <c r="Q34">
+        <v>2022</v>
+      </c>
+      <c r="R34" t="str">
+        <v>Operational — 4 lane</v>
+      </c>
+      <c r="S34" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T34" t="str">
+        <v>Partial</v>
+      </c>
+      <c r="U34" t="str">
+        <v>Kolhapur–Sangli industrial link</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>SH-34</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Nashik</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Malegaon</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Nashik</v>
+      </c>
+      <c r="E35">
+        <v>90</v>
+      </c>
+      <c r="F35" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G35" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H35" t="str">
+        <v>Strengthening 2018–2021</v>
+      </c>
+      <c r="I35">
+        <v>2022</v>
+      </c>
+      <c r="J35" t="str">
+        <v>Bituminous overlay</v>
+      </c>
+      <c r="K35" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L35" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M35" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N35" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O35" t="str">
+        <v>~₹115 Cr</v>
+      </c>
+      <c r="P35">
+        <v>2018</v>
+      </c>
+      <c r="Q35">
+        <v>2021</v>
+      </c>
+      <c r="R35" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S35" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T35" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U35" t="str">
+        <v>Malegaon textile sector access</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>SH-36</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Panvel</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Alibaug</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Raigad</v>
+      </c>
+      <c r="E36">
+        <v>50</v>
+      </c>
+      <c r="F36" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G36" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H36" t="str">
+        <v>Widening 2020–2023 (Mumbai coastal zone)</v>
+      </c>
+      <c r="I36">
+        <v>2023</v>
+      </c>
+      <c r="J36" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K36" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L36" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M36" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N36" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O36" t="str">
+        <v>~₹95 Cr</v>
+      </c>
+      <c r="P36">
+        <v>2020</v>
+      </c>
+      <c r="Q36">
+        <v>2023</v>
+      </c>
+      <c r="R36" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S36" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T36" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U36" t="str">
+        <v>Konkan coastal access</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>SH-37</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Thane</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Shahapur</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Thane</v>
+      </c>
+      <c r="E37">
+        <v>80</v>
+      </c>
+      <c r="F37" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G37" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H37" t="str">
+        <v>Resurfacing 2022</v>
+      </c>
+      <c r="I37">
+        <v>2022</v>
+      </c>
+      <c r="J37" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K37" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L37" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M37" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N37" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O37" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="P37" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="Q37" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="R37" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S37" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T37" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U37" t="str">
+        <v>Part of MMR hinterland network</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>SH-38</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Vasai</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Bhiwandi</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Palghar, Thane</v>
+      </c>
+      <c r="E38">
+        <v>45</v>
+      </c>
+      <c r="F38" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G38" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H38" t="str">
+        <v>Strengthening 2019–2021</v>
+      </c>
+      <c r="I38">
+        <v>2022</v>
+      </c>
+      <c r="J38" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K38" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L38" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M38" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N38" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O38" t="str">
+        <v>~₹68 Cr</v>
+      </c>
+      <c r="P38">
+        <v>2019</v>
+      </c>
+      <c r="Q38">
+        <v>2021</v>
+      </c>
+      <c r="R38" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S38" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T38" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U38" t="str">
+        <v>Logistics hub access</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>SH-39</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Hingoli</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Nanded</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Hingoli, Nanded</v>
+      </c>
+      <c r="E39">
+        <v>70</v>
+      </c>
+      <c r="F39" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G39" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H39" t="str">
+        <v>Resurfacing 2021</v>
+      </c>
+      <c r="I39">
+        <v>2021</v>
+      </c>
+      <c r="J39" t="str">
+        <v>Bituminous overlay</v>
+      </c>
+      <c r="K39" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L39" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M39" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N39" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O39" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="P39" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="Q39" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="R39" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S39" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T39" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U39" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>SH-40</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Aurangabad</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Jalgaon</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Aurangabad, Jalgaon</v>
+      </c>
+      <c r="E40">
+        <v>180</v>
+      </c>
+      <c r="F40" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G40" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H40" t="str">
+        <v>Widening 2016–2020</v>
+      </c>
+      <c r="I40">
+        <v>2022</v>
+      </c>
+      <c r="J40" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K40" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L40" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M40" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N40" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O40" t="str">
+        <v>~₹235 Cr</v>
+      </c>
+      <c r="P40">
+        <v>2016</v>
+      </c>
+      <c r="Q40">
+        <v>2020</v>
+      </c>
+      <c r="R40" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S40" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T40" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U40" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>SH-43</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Kolhapur</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Ichalkaranji</v>
+      </c>
+      <c r="D41" t="str">
+        <v>Kolhapur</v>
+      </c>
+      <c r="E41">
+        <v>35</v>
+      </c>
+      <c r="F41" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G41" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H41" t="str">
+        <v>4-laning 2019–2022</v>
+      </c>
+      <c r="I41">
+        <v>2022</v>
+      </c>
+      <c r="J41" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K41" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L41" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M41" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N41" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O41" t="str">
+        <v>~₹55 Cr</v>
+      </c>
+      <c r="P41">
+        <v>2019</v>
+      </c>
+      <c r="Q41">
+        <v>2022</v>
+      </c>
+      <c r="R41" t="str">
+        <v>Operational — 4 lane</v>
+      </c>
+      <c r="S41" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T41" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U41" t="str">
+        <v>Textile city access road</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>SH-44</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Nandurbar</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Dhule</v>
+      </c>
+      <c r="D42" t="str">
+        <v>Nandurbar, Dhule</v>
+      </c>
+      <c r="E42">
+        <v>70</v>
+      </c>
+      <c r="F42" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G42" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H42" t="str">
+        <v>Strengthening 2018–2020</v>
+      </c>
+      <c r="I42">
+        <v>2021</v>
+      </c>
+      <c r="J42" t="str">
+        <v>Bituminous overlay</v>
+      </c>
+      <c r="K42" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L42" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M42" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N42" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O42" t="str">
+        <v>~₹88 Cr</v>
+      </c>
+      <c r="P42">
+        <v>2018</v>
+      </c>
+      <c r="Q42">
+        <v>2020</v>
+      </c>
+      <c r="R42" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S42" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T42" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U42" t="str">
+        <v>Tribal belt — Nandurbar Adivasi area</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>SH-45</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Ratnagiri</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Lanja</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Ratnagiri</v>
+      </c>
+      <c r="E43">
+        <v>50</v>
+      </c>
+      <c r="F43" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G43" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H43" t="str">
+        <v>Resurfacing 2021–2023</v>
+      </c>
+      <c r="I43">
+        <v>2023</v>
+      </c>
+      <c r="J43" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K43" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L43" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M43" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N43" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O43" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="P43" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="Q43" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="R43" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S43" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T43" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U43" t="str">
+        <v>Konkan rural connectivity</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>SH-47</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Satara</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Wai</v>
+      </c>
+      <c r="D44" t="str">
+        <v>Satara</v>
+      </c>
+      <c r="E44">
+        <v>30</v>
+      </c>
+      <c r="F44" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G44" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H44" t="str">
+        <v>Resurfacing 2020</v>
+      </c>
+      <c r="I44">
+        <v>2020</v>
+      </c>
+      <c r="J44" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K44" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L44" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M44" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N44" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O44" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="P44" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="Q44" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="R44" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S44" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T44" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U44" t="str">
+        <v>Panchgani/Mahabaleshwar access route</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>SH-48</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Pune</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Ahmednagar</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Pune, Ahmednagar</v>
+      </c>
+      <c r="E45">
+        <v>100</v>
+      </c>
+      <c r="F45" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G45" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H45" t="str">
+        <v>Widening 2016–2019</v>
+      </c>
+      <c r="I45">
+        <v>2022</v>
+      </c>
+      <c r="J45" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K45" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L45" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M45" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N45" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O45" t="str">
+        <v>~₹140 Cr</v>
+      </c>
+      <c r="P45">
+        <v>2016</v>
+      </c>
+      <c r="Q45">
+        <v>2019</v>
+      </c>
+      <c r="R45" t="str">
+        <v>Operational — 2/4 lane</v>
+      </c>
+      <c r="S45" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T45" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U45" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>SH-49</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Sangli</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Miraj</v>
+      </c>
+      <c r="D46" t="str">
+        <v>Sangli</v>
+      </c>
+      <c r="E46">
+        <v>15</v>
+      </c>
+      <c r="F46" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G46" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H46" t="str">
+        <v>4-laning 2020–2022</v>
+      </c>
+      <c r="I46">
+        <v>2022</v>
+      </c>
+      <c r="J46" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K46" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L46" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M46" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N46" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O46" t="str">
+        <v>~₹28 Cr</v>
+      </c>
+      <c r="P46">
+        <v>2020</v>
+      </c>
+      <c r="Q46">
+        <v>2022</v>
+      </c>
+      <c r="R46" t="str">
+        <v>Operational — 4 lane (urban)</v>
+      </c>
+      <c r="S46" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T46" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U46" t="str">
+        <v>Twin city connector</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>SH-50</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Solapur</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Pandharpur</v>
+      </c>
+      <c r="D47" t="str">
+        <v>Solapur</v>
+      </c>
+      <c r="E47">
+        <v>70</v>
+      </c>
+      <c r="F47" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G47" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H47" t="str">
+        <v>Pilgrimage corridor upgradation 2019–2022</v>
+      </c>
+      <c r="I47">
+        <v>2023</v>
+      </c>
+      <c r="J47" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K47" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L47" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M47" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N47" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O47" t="str">
+        <v>~₹95 Cr</v>
+      </c>
+      <c r="P47">
+        <v>2019</v>
+      </c>
+      <c r="Q47">
+        <v>2022</v>
+      </c>
+      <c r="R47" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S47" t="str">
+        <v>Maharashtra PWD; Maharashtra Tourism</v>
+      </c>
+      <c r="T47" t="str">
+        <v>Partial</v>
+      </c>
+      <c r="U47" t="str">
+        <v>Pandharpur Wari pilgrimage route; handles millions of pilgrims annually</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>SH-52</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Parbhani</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Nanded</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Parbhani, Hingoli, Nanded</v>
+      </c>
+      <c r="E48">
+        <v>90</v>
+      </c>
+      <c r="F48" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G48" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H48" t="str">
+        <v>Strengthening 2017–2020</v>
+      </c>
+      <c r="I48">
+        <v>2021</v>
+      </c>
+      <c r="J48" t="str">
+        <v>Bituminous overlay</v>
+      </c>
+      <c r="K48" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L48" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M48" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N48" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O48" t="str">
+        <v>~₹112 Cr</v>
+      </c>
+      <c r="P48">
+        <v>2017</v>
+      </c>
+      <c r="Q48">
+        <v>2020</v>
+      </c>
+      <c r="R48" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S48" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T48" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U48" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>SH-53</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Chandrapur</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Nagpur</v>
+      </c>
+      <c r="D49" t="str">
+        <v>Chandrapur, Nagpur</v>
+      </c>
+      <c r="E49">
+        <v>120</v>
+      </c>
+      <c r="F49" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G49" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H49" t="str">
+        <v>Widening 2018–2022</v>
+      </c>
+      <c r="I49">
+        <v>2022</v>
+      </c>
+      <c r="J49" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K49" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L49" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M49" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N49" t="str">
+        <v>PNC Infratech (partial)</v>
+      </c>
+      <c r="O49" t="str">
+        <v>~₹165 Cr</v>
+      </c>
+      <c r="P49">
+        <v>2018</v>
+      </c>
+      <c r="Q49">
+        <v>2022</v>
+      </c>
+      <c r="R49" t="str">
+        <v>Operational — 2/4 lane</v>
+      </c>
+      <c r="S49" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T49" t="str">
+        <v>Partial</v>
+      </c>
+      <c r="U49" t="str">
+        <v>Chandrapur coal/thermal power region</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>SH-55</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Kolhapur</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Ajra</v>
+      </c>
+      <c r="D50" t="str">
+        <v>Kolhapur</v>
+      </c>
+      <c r="E50">
+        <v>80</v>
+      </c>
+      <c r="F50" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G50" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H50" t="str">
+        <v>Resurfacing 2021–2022</v>
+      </c>
+      <c r="I50">
+        <v>2022</v>
+      </c>
+      <c r="J50" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K50" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L50" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M50" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N50" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O50" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="P50" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="Q50" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="R50" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S50" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T50" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U50" t="str">
+        <v>Konkan hinterland access</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>SH-60</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Pune</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Mumbai (via Khopoli Old Highway)</v>
+      </c>
+      <c r="D51" t="str">
+        <v>Pune, Raigad</v>
+      </c>
+      <c r="E51">
+        <v>120</v>
+      </c>
+      <c r="F51" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G51" t="str">
+        <v>Maharashtra State Road Development Corporation (MSRDC)</v>
+      </c>
+      <c r="H51" t="str">
+        <v>Maintained as alternative to Expressway; resurfacing 2022</v>
+      </c>
+      <c r="I51">
+        <v>2022</v>
+      </c>
+      <c r="J51" t="str">
+        <v>Bituminous overlay</v>
+      </c>
+      <c r="K51" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L51" t="str">
+        <v>MD, MSRDC; CE, Maharashtra PWD</v>
+      </c>
+      <c r="M51" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N51" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O51" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="P51" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="Q51" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="R51" t="str">
+        <v>Operational — 4 lane</v>
+      </c>
+      <c r="S51" t="str">
+        <v>MSRDC; Maharashtra PWD</v>
+      </c>
+      <c r="T51" t="str">
+        <v>Partial</v>
+      </c>
+      <c r="U51" t="str">
+        <v>Original Pune–Mumbai highway via Khandala Ghats; still heavily used by trucks and locals</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>SH-70</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Nagpur</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Hinganghat</v>
+      </c>
+      <c r="D52" t="str">
+        <v>Nagpur, Wardha</v>
+      </c>
+      <c r="E52">
+        <v>85</v>
+      </c>
+      <c r="F52" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G52" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H52" t="str">
+        <v>Strengthening 2019–2021</v>
+      </c>
+      <c r="I52">
+        <v>2021</v>
+      </c>
+      <c r="J52" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K52" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L52" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M52" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N52" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O52" t="str">
+        <v>~₹108 Cr</v>
+      </c>
+      <c r="P52">
+        <v>2019</v>
+      </c>
+      <c r="Q52">
+        <v>2021</v>
+      </c>
+      <c r="R52" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S52" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T52" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U52" t="str">
+        <v>Cotton processing zone</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>SH-72</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Kolhapur</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Ratnagiri</v>
+      </c>
+      <c r="D53" t="str">
+        <v>Kolhapur, Sindhudurg, Ratnagiri</v>
+      </c>
+      <c r="E53">
+        <v>210</v>
+      </c>
+      <c r="F53" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G53" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H53" t="str">
+        <v>Widening 2016–2021</v>
+      </c>
+      <c r="I53">
+        <v>2022</v>
+      </c>
+      <c r="J53" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K53" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L53" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M53" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N53" t="str">
+        <v>IRB Infrastructure (partial)</v>
+      </c>
+      <c r="O53" t="str">
+        <v>~₹320 Cr</v>
+      </c>
+      <c r="P53">
+        <v>2016</v>
+      </c>
+      <c r="Q53">
+        <v>2021</v>
+      </c>
+      <c r="R53" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S53" t="str">
+        <v>Maharashtra PWD; IRB Infra news</v>
+      </c>
+      <c r="T53" t="str">
+        <v>Partial</v>
+      </c>
+      <c r="U53" t="str">
+        <v>Long coastal/ghats corridor; multiple tunnels proposed</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>SH-140</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Panvel</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Mumbai (Trans-Harbour)</v>
+      </c>
+      <c r="D54" t="str">
+        <v>Raigad, Mumbai</v>
+      </c>
+      <c r="E54">
+        <v>60</v>
+      </c>
+      <c r="F54" t="str">
+        <v>Maharashtra State Road Development Corporation (MSRDC)</v>
+      </c>
+      <c r="G54" t="str">
+        <v>Maharashtra State Road Development Corporation (MSRDC)</v>
+      </c>
+      <c r="H54" t="str">
+        <v>Maintained as part of Mumbai Metro region roads</v>
+      </c>
+      <c r="I54">
+        <v>2022</v>
+      </c>
+      <c r="J54" t="str">
+        <v>Resurfacing</v>
+      </c>
+      <c r="K54" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L54" t="str">
+        <v>MD, MSRDC</v>
+      </c>
+      <c r="M54" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N54" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O54" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="P54" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="Q54" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="R54" t="str">
+        <v>Operational — 4/6 lane (urban)</v>
+      </c>
+      <c r="S54" t="str">
+        <v>MSRDC</v>
+      </c>
+      <c r="T54" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U54" t="str">
+        <v>Part of Mumbai Metropolitan Region (MMR) road network</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>SH-149</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Nashik</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Shirdi</v>
+      </c>
+      <c r="D55" t="str">
+        <v>Nashik, Ahmednagar</v>
+      </c>
+      <c r="E55">
+        <v>80</v>
+      </c>
+      <c r="F55" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G55" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H55" t="str">
+        <v>4-laning 2018–2021 (pilgrimage corridor)</v>
+      </c>
+      <c r="I55">
+        <v>2022</v>
+      </c>
+      <c r="J55" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K55" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L55" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M55" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N55" t="str">
+        <v>Dilip Buildcon</v>
+      </c>
+      <c r="O55" t="str">
+        <v>~₹115 Cr</v>
+      </c>
+      <c r="P55">
+        <v>2018</v>
+      </c>
+      <c r="Q55">
+        <v>2021</v>
+      </c>
+      <c r="R55" t="str">
+        <v>Operational — 4 lane</v>
+      </c>
+      <c r="S55" t="str">
+        <v>Maharashtra PWD; PIB 2021</v>
+      </c>
+      <c r="T55" t="str">
+        <v>Partial</v>
+      </c>
+      <c r="U55" t="str">
+        <v>Kumbh Mela pilgrimage route (Nashik); Shirdi Sai Baba temple access</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>SH-166</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Aurangabad</v>
+      </c>
+      <c r="C56" t="str">
+        <v>Solapur</v>
+      </c>
+      <c r="D56" t="str">
+        <v>Aurangabad, Beed, Osmanabad, Solapur</v>
+      </c>
+      <c r="E56">
+        <v>250</v>
+      </c>
+      <c r="F56" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G56" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H56" t="str">
+        <v>Strengthening 2015–2019</v>
+      </c>
+      <c r="I56">
+        <v>2022</v>
+      </c>
+      <c r="J56" t="str">
+        <v>Periodic renewal</v>
+      </c>
+      <c r="K56" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L56" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M56" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N56" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O56" t="str">
+        <v>~₹345 Cr</v>
+      </c>
+      <c r="P56">
+        <v>2015</v>
+      </c>
+      <c r="Q56">
+        <v>2019</v>
+      </c>
+      <c r="R56" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S56" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T56" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U56" t="str">
+        <v>Important Marathwada–Solapur corridor</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>SH-190</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Kolhapur</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Malvan</v>
+      </c>
+      <c r="D57" t="str">
+        <v>Kolhapur, Sindhudurg</v>
+      </c>
+      <c r="E57">
+        <v>130</v>
+      </c>
+      <c r="F57" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G57" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H57" t="str">
+        <v>Konkan coastal road improvements 2019–2022</v>
+      </c>
+      <c r="I57">
+        <v>2022</v>
+      </c>
+      <c r="J57" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K57" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L57" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M57" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N57" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O57" t="str">
+        <v>~₹175 Cr</v>
+      </c>
+      <c r="P57">
+        <v>2019</v>
+      </c>
+      <c r="Q57">
+        <v>2022</v>
+      </c>
+      <c r="R57" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S57" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T57" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U57" t="str">
+        <v>Konkan coastal tourism corridor; Malvan is a heritage and beach tourism destination</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>SH-204</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Nagpur</v>
+      </c>
+      <c r="C58" t="str">
+        <v>Butibori MIDC</v>
+      </c>
+      <c r="D58" t="str">
+        <v>Nagpur</v>
+      </c>
+      <c r="E58">
+        <v>35</v>
+      </c>
+      <c r="F58" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G58" t="str">
+        <v>MIDC / Maharashtra PWD</v>
+      </c>
+      <c r="H58" t="str">
+        <v>MIDC access road upgradation 2020–2022</v>
+      </c>
+      <c r="I58">
+        <v>2022</v>
+      </c>
+      <c r="J58" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K58" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L58" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M58" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N58" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O58" t="str">
+        <v>~₹52 Cr</v>
+      </c>
+      <c r="P58">
+        <v>2020</v>
+      </c>
+      <c r="Q58">
+        <v>2022</v>
+      </c>
+      <c r="R58" t="str">
+        <v>Operational — 4 lane</v>
+      </c>
+      <c r="S58" t="str">
+        <v>MIDC; Maharashtra PWD</v>
+      </c>
+      <c r="T58" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U58" t="str">
+        <v>Butibori is one of Asia's largest industrial zones</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>SH-216</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Satara</v>
+      </c>
+      <c r="C59" t="str">
+        <v>Koregaon</v>
+      </c>
+      <c r="D59" t="str">
+        <v>Satara</v>
+      </c>
+      <c r="E59">
+        <v>30</v>
+      </c>
+      <c r="F59" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G59" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H59" t="str">
+        <v>Resurfacing 2021</v>
+      </c>
+      <c r="I59">
+        <v>2021</v>
+      </c>
+      <c r="J59" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K59" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L59" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M59" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N59" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O59" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="P59" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="Q59" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="R59" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S59" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T59" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U59" t="str">
+        <v>Koregaon–Bhima historical site access road</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>SH-220</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Pune</v>
+      </c>
+      <c r="C60" t="str">
+        <v>Saswad</v>
+      </c>
+      <c r="D60" t="str">
+        <v>Pune</v>
+      </c>
+      <c r="E60">
+        <v>35</v>
+      </c>
+      <c r="F60" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G60" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H60" t="str">
+        <v>4-laning 2019–2021</v>
+      </c>
+      <c r="I60">
+        <v>2022</v>
+      </c>
+      <c r="J60" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K60" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L60" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M60" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N60" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O60" t="str">
+        <v>~₹55 Cr</v>
+      </c>
+      <c r="P60">
+        <v>2019</v>
+      </c>
+      <c r="Q60">
+        <v>2021</v>
+      </c>
+      <c r="R60" t="str">
+        <v>Operational — 4 lane (peri-urban)</v>
+      </c>
+      <c r="S60" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T60" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U60" t="str">
+        <v>Saswad — growing industrial/logistics zone near Pune</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>SH-249</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Nagpur</v>
+      </c>
+      <c r="C61" t="str">
+        <v>Ramtek</v>
+      </c>
+      <c r="D61" t="str">
+        <v>Nagpur</v>
+      </c>
+      <c r="E61">
+        <v>45</v>
+      </c>
+      <c r="F61" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G61" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H61" t="str">
+        <v>Pilgrimage road improvements 2021–2023</v>
+      </c>
+      <c r="I61">
+        <v>2023</v>
+      </c>
+      <c r="J61" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K61" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L61" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M61" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N61" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O61" t="str">
+        <v>~₹62 Cr</v>
+      </c>
+      <c r="P61">
+        <v>2021</v>
+      </c>
+      <c r="Q61">
+        <v>2023</v>
+      </c>
+      <c r="R61" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S61" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T61" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U61" t="str">
+        <v>Ramtek — significant religious site associated with Kalidasa and Lord Ram</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>SH-261</v>
+      </c>
+      <c r="B62" t="str">
+        <v>Nashik</v>
+      </c>
+      <c r="C62" t="str">
+        <v>Ozar</v>
+      </c>
+      <c r="D62" t="str">
+        <v>Nashik</v>
+      </c>
+      <c r="E62">
+        <v>30</v>
+      </c>
+      <c r="F62" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G62" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H62" t="str">
+        <v>Industrial access upgrade 2020–2022</v>
+      </c>
+      <c r="I62">
+        <v>2022</v>
+      </c>
+      <c r="J62" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K62" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L62" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M62" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N62" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O62" t="str">
+        <v>~₹48 Cr</v>
+      </c>
+      <c r="P62">
+        <v>2020</v>
+      </c>
+      <c r="Q62">
+        <v>2022</v>
+      </c>
+      <c r="R62" t="str">
+        <v>Operational — 4 lane</v>
+      </c>
+      <c r="S62" t="str">
+        <v>Maharashtra PWD</v>
+      </c>
+      <c r="T62" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U62" t="str">
+        <v>Ozar Airport and HAL/Defence facility access road</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>SH-272</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Kolhapur</v>
+      </c>
+      <c r="C63" t="str">
+        <v>Panhala</v>
+      </c>
+      <c r="D63" t="str">
+        <v>Kolhapur</v>
+      </c>
+      <c r="E63">
+        <v>22</v>
+      </c>
+      <c r="F63" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="G63" t="str">
+        <v>Maharashtra Public Works Department (PWD)</v>
+      </c>
+      <c r="H63" t="str">
+        <v>Tourism road improvement 2020–2022</v>
+      </c>
+      <c r="I63">
+        <v>2022</v>
+      </c>
+      <c r="J63" t="str">
+        <v>Overlay</v>
+      </c>
+      <c r="K63" t="str">
+        <v>Ravindra Chavan, PWD Minister, Maharashtra (BJP/Mahayuti Govt)</v>
+      </c>
+      <c r="L63" t="str">
+        <v>Chief Engineer, Maharashtra PWD (file RTI for current officer name)</v>
+      </c>
+      <c r="M63" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="N63" t="str">
+        <v>Not available in public domain — file RTI at rtionline.gov.in</v>
+      </c>
+      <c r="O63" t="str">
+        <v>~₹32 Cr</v>
+      </c>
+      <c r="P63">
+        <v>2020</v>
+      </c>
+      <c r="Q63">
+        <v>2022</v>
+      </c>
+      <c r="R63" t="str">
+        <v>Operational — 2 lane</v>
+      </c>
+      <c r="S63" t="str">
+        <v>Maharashtra PWD; Maharashtra Tourism</v>
+      </c>
+      <c r="T63" t="str">
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="U63" t="str">
+        <v>Panhala Fort — historic Maratha fort; major tourism site</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:U63"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D13"/>
   <cols>
     <col min="1" max="1" width="53.83203125" customWidth="1"/>
@@ -5269,7 +9399,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F7"/>
   <cols>
@@ -5428,9 +9558,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:B30"/>
   <cols>
     <col min="1" max="1" width="70.83203125" customWidth="1"/>
     <col min="2" max="2" width="40.83203125" customWidth="1"/>
@@ -5451,7 +9581,7 @@
         <v>Generated</v>
       </c>
       <c r="B3" t="str">
-        <v>23/5/2026</v>
+        <v>24/5/2026</v>
       </c>
     </row>
     <row r="4">
@@ -5472,133 +9602,133 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v/>
+        <v>Total MH SH rows</v>
+      </c>
+      <c r="B6">
+        <v>62</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>DATA QUALITY LEGEND</v>
+        <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>High Confidence</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Data verified against NHAI/MoRTH/CAG official publications</v>
+        <v>DATA QUALITY LEGEND</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Partial</v>
+        <v>High Confidence</v>
       </c>
       <c r="B9" t="str">
-        <v>Route &amp; authority confirmed; some admin details estimated from news/reports</v>
+        <v>Data verified against NHAI/MoRTH/CAG official publications</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Template Only - RTI Required</v>
+        <v>Partial</v>
       </c>
       <c r="B10" t="str">
-        <v>Route confirmed; most fields need RTI to get exact data</v>
+        <v>Route &amp; authority confirmed; some admin details estimated from news/reports</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v/>
+        <v>Template Only - RTI Required</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Route confirmed; most fields need RTI to get exact data</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>KEY ABBREVIATIONS</v>
+        <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>NHAI</v>
-      </c>
-      <c r="B13" t="str">
-        <v>National Highways Authority of India</v>
+        <v>KEY ABBREVIATIONS</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>MoRTH</v>
+        <v>NHAI</v>
       </c>
       <c r="B14" t="str">
-        <v>Ministry of Road Transport &amp; Highways</v>
+        <v>National Highways Authority of India</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>NHIDCL</v>
+        <v>MoRTH</v>
       </c>
       <c r="B15" t="str">
-        <v>National Highways &amp; Infrastructure Development Corporation</v>
+        <v>Ministry of Road Transport &amp; Highways</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>NHDP</v>
+        <v>NHIDCL</v>
       </c>
       <c r="B16" t="str">
-        <v>National Highway Development Programme (Phases I–VII)</v>
+        <v>National Highways &amp; Infrastructure Development Corporation</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>TNHD</v>
+        <v>NHDP</v>
       </c>
       <c r="B17" t="str">
-        <v>Tamil Nadu Highways Department</v>
+        <v>National Highway Development Programme (Phases I–VII)</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>TNRSP</v>
+        <v>TNHD</v>
       </c>
       <c r="B18" t="str">
-        <v>Tamil Nadu Road Sector Project (World Bank funded)</v>
+        <v>Tamil Nadu Highways Department</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>DG(RD)</v>
+        <v>TNRSP</v>
       </c>
       <c r="B19" t="str">
-        <v>Director General, Road Development (MoRTH)</v>
+        <v>Tamil Nadu Road Sector Project (World Bank funded)</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>SE</v>
+        <v>DG(RD)</v>
       </c>
       <c r="B20" t="str">
-        <v>Superintending Engineer</v>
+        <v>Director General, Road Development (MoRTH)</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v/>
+        <v>SE</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Superintending Engineer</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>IMPORTANT NOTE</v>
+        <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Fields marked "Not available in public domain — file RTI" genuinely cannot be found in any</v>
-      </c>
-      <c r="B23" t="str">
-        <v/>
+        <v>IMPORTANT NOTE</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>free public database. Lead engineer names, exact repair dates, and stretch-level contractor</v>
+        <v>Fields marked "Not available in public domain — file RTI" genuinely cannot be found in any</v>
       </c>
       <c r="B24" t="str">
         <v/>
@@ -5606,7 +9736,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>details require RTI filing or official tender document requests. See RTI Guide sheet.</v>
+        <v>free public database. Lead engineer names, exact repair dates, and stretch-level contractor</v>
       </c>
       <c r="B25" t="str">
         <v/>
@@ -5614,20 +9744,20 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
+        <v>details require RTI filing or official tender document requests. See RTI Guide sheet.</v>
+      </c>
+      <c r="B26" t="str">
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>TO GET REMAINING DATA — use RTI Online portal: https://rtionline.gov.in/ (₹10 fee, 30 days)</v>
-      </c>
-      <c r="B27" t="str">
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Or check eProcure: https://eprocure.gov.in/ for tender award details</v>
+        <v>TO GET REMAINING DATA — use RTI Online portal: https://rtionline.gov.in/ (₹10 fee, 30 days)</v>
       </c>
       <c r="B28" t="str">
         <v/>
@@ -5635,15 +9765,23 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Or check PFMS: https://pfms.nic.in/ for government expenditure data</v>
+        <v>Or check eProcure: https://eprocure.gov.in/ for tender award details</v>
       </c>
       <c r="B29" t="str">
         <v/>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>Or check PFMS: https://pfms.nic.in/ for government expenditure data</v>
+      </c>
+      <c r="B30" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B29"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B30"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>